<commit_message>
this is what I get for not pushing for three days
</commit_message>
<xml_diff>
--- a/week-02/Ex2A_events_normalized.xlsx
+++ b/week-02/Ex2A_events_normalized.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30002"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30006"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://reliablecollaboration.sharepoint.com/sites/Customers/Shared Documents/cust-pluralsight/YearUpSpring2026_DataAnalytics/DA course material/Week 2 - SQL Part 1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{849D3C42-6060-41DF-9A16-CC23B270F4DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4387552D-8ABC-4B04-B5B4-8F20FE0D5179}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1035" yWindow="630" windowWidth="38700" windowHeight="15345" xr2:uid="{5091876E-AF08-41C4-B976-D2AB9D8B455C}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="132">
   <si>
     <t>It said It was up to 3NF</t>
   </si>
@@ -415,6 +415,9 @@
     <t>Category Code</t>
   </si>
   <si>
+    <t>Art</t>
+  </si>
+  <si>
     <t>Music</t>
   </si>
   <si>
@@ -431,9 +434,6 @@
   </si>
   <si>
     <t>Film</t>
-  </si>
-  <si>
-    <t>Art</t>
   </si>
 </sst>
 </file>
@@ -1322,7 +1322,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FA38BEC-78EC-44DC-83F3-AA711D021920}">
-  <dimension ref="A1:G79"/>
+  <dimension ref="A1:G77"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="27.28515625" style="5" bestFit="1" customWidth="1"/>
@@ -2046,12 +2046,12 @@
         <v>125</v>
       </c>
       <c r="C69">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70" spans="1:3">
       <c r="B70" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C70">
         <v>7</v>
@@ -2059,7 +2059,7 @@
     </row>
     <row r="71" spans="1:3">
       <c r="B71" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C71">
         <v>2</v>
@@ -2067,7 +2067,7 @@
     </row>
     <row r="72" spans="1:3">
       <c r="B72" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C72">
         <v>3</v>
@@ -2075,7 +2075,7 @@
     </row>
     <row r="73" spans="1:3">
       <c r="B73" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C73">
         <v>6</v>
@@ -2083,7 +2083,7 @@
     </row>
     <row r="74" spans="1:3">
       <c r="B74" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C74">
         <v>4</v>
@@ -2091,7 +2091,7 @@
     </row>
     <row r="75" spans="1:3">
       <c r="B75" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C75">
         <v>5</v>
@@ -2099,7 +2099,7 @@
     </row>
     <row r="76" spans="1:3">
       <c r="B76" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C76">
         <v>3</v>
@@ -2107,26 +2107,10 @@
     </row>
     <row r="77" spans="1:3">
       <c r="B77" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C77">
         <v>7</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3">
-      <c r="B78" t="s">
-        <v>126</v>
-      </c>
-      <c r="C78">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3">
-      <c r="B79" t="s">
-        <v>131</v>
-      </c>
-      <c r="C79">
-        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2501,7 +2485,7 @@
         <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E2">
         <v>7</v>
@@ -2533,7 +2517,7 @@
         <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E3">
         <v>7</v>
@@ -2565,7 +2549,7 @@
         <v>17</v>
       </c>
       <c r="D4" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E4">
         <v>2</v>
@@ -2597,7 +2581,7 @@
         <v>20</v>
       </c>
       <c r="D5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E5">
         <v>3</v>
@@ -2629,7 +2613,7 @@
         <v>24</v>
       </c>
       <c r="D6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E6">
         <v>6</v>
@@ -2661,7 +2645,7 @@
         <v>20</v>
       </c>
       <c r="D7" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E7">
         <v>4</v>
@@ -2693,7 +2677,7 @@
         <v>28</v>
       </c>
       <c r="D8" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E8">
         <v>5</v>
@@ -2725,7 +2709,7 @@
         <v>32</v>
       </c>
       <c r="D9" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E9">
         <v>3</v>
@@ -2757,7 +2741,7 @@
         <v>9</v>
       </c>
       <c r="D10" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E10">
         <v>7</v>
@@ -2789,7 +2773,7 @@
         <v>36</v>
       </c>
       <c r="D11" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E11">
         <v>2</v>
@@ -2821,7 +2805,7 @@
         <v>38</v>
       </c>
       <c r="D12" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2884,12 +2868,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="ced60a7f-99b1-48d2-b555-34851c8026ae" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9e0b35a9-e6cb-436b-81d4-4440ba439ca5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3134,18 +3120,16 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="ced60a7f-99b1-48d2-b555-34851c8026ae" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9e0b35a9-e6cb-436b-81d4-4440ba439ca5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D48FB9E6-6DE3-40FB-81F7-677295638F7C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1EE6EC55-B0E7-4ACE-A5DA-E03DCA4973DE}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3153,5 +3137,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1EE6EC55-B0E7-4ACE-A5DA-E03DCA4973DE}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D48FB9E6-6DE3-40FB-81F7-677295638F7C}"/>
 </file>
</xml_diff>